<commit_message>
[Progress] ใส่ function print แล้ว อื่นๆ...
[Lacking] ขาดตัวจัดการ state,
[issue] memory บน chrome keep raising
</commit_message>
<xml_diff>
--- a/projects/Finance/inv_example.xlsx
+++ b/projects/Finance/inv_example.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BCP_27\Documents\GitHub\Python\projects\Finance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B34A213-ED70-4461-A872-3F1B5DD4FC28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D630CD20-991E-49B6-B184-B93D0DD45B7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31590" yWindow="1560" windowWidth="19425" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32145" yWindow="795" windowWidth="19425" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,33 +28,57 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
   <si>
     <t>INVOICE_NO</t>
   </si>
   <si>
-    <t>B0183-W11-2408280020</t>
-  </si>
-  <si>
-    <t>B0183-W11-2408280021</t>
-  </si>
-  <si>
-    <t>B0183-W14-2408280008</t>
-  </si>
-  <si>
-    <t>B0183-w12-2408280004</t>
-  </si>
-  <si>
-    <t>B0183-W11-2408280022</t>
-  </si>
-  <si>
-    <t>B0183-W14-2408280009</t>
-  </si>
-  <si>
-    <t>B0183-W14-2408280010</t>
-  </si>
-  <si>
-    <t>B0183-w12-2408280005</t>
+    <t>B0183-W14-2408280011</t>
+  </si>
+  <si>
+    <t>B0183-W11-2408280023</t>
+  </si>
+  <si>
+    <t>B0183-w12-2408280006</t>
+  </si>
+  <si>
+    <t>B0183-w12-2408280007</t>
+  </si>
+  <si>
+    <t>B0183-w12-2408280008</t>
+  </si>
+  <si>
+    <t>B0183-w12-2408280009</t>
+  </si>
+  <si>
+    <t>B0183-W14-2408280014</t>
+  </si>
+  <si>
+    <t>B0183-W14-2408280023</t>
+  </si>
+  <si>
+    <t>B0183-W14-2408280029</t>
+  </si>
+  <si>
+    <t>B0183-W14-2408280030</t>
+  </si>
+  <si>
+    <t>B0183-W14-2408280031</t>
+  </si>
+  <si>
+    <t>B0183-w12-2408280010</t>
+  </si>
+  <si>
+    <t>B0183-W14-2408280037</t>
+  </si>
+  <si>
+    <t>B0183-W14-2408280038</t>
+  </si>
+  <si>
+    <t>B0183-W14-2408280039</t>
+  </si>
+  <si>
+    <t>B0183-W14-2408280040</t>
   </si>
 </sst>
 </file>
@@ -90,8 +114,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -297,103 +322,103 @@
       </c>
     </row>
     <row r="2" spans="1:1">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
-      <c r="A4" t="s">
+    <row r="6" spans="1:1">
+      <c r="A6" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
-      <c r="A5" t="s">
+    <row r="7" spans="1:1">
+      <c r="A7" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:1">
-      <c r="A6" t="s">
+    <row r="8" spans="1:1">
+      <c r="A8" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:1">
-      <c r="A7" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1">
-      <c r="A8" t="s">
-        <v>3</v>
-      </c>
-    </row>
     <row r="9" spans="1:1">
-      <c r="A9" t="s">
+      <c r="A9" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:1">
-      <c r="A10" t="s">
+      <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:1">
-      <c r="A11" t="s">
-        <v>5</v>
+      <c r="A11" s="1" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:1">
-      <c r="A12" t="s">
-        <v>5</v>
+      <c r="A12" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:1">
-      <c r="A13" t="s">
-        <v>6</v>
+      <c r="A13" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="14" spans="1:1">
-      <c r="A14" t="s">
-        <v>6</v>
+      <c r="A14" s="1" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:1">
-      <c r="A15" t="s">
-        <v>6</v>
+      <c r="A15" s="1" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:1">
-      <c r="A16" t="s">
-        <v>7</v>
+      <c r="A16" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="17" spans="1:1">
-      <c r="A17" t="s">
-        <v>8</v>
+      <c r="A17" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="18" spans="1:1">
-      <c r="A18" t="s">
-        <v>8</v>
+      <c r="A18" s="1" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="19" spans="1:1">
-      <c r="A19" t="s">
-        <v>8</v>
+      <c r="A19" s="1" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:1">
-      <c r="A20" t="s">
-        <v>8</v>
+      <c r="A20" s="1" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="21" spans="1:1">
-      <c r="A21" t="s">
-        <v>8</v>
+      <c r="A21" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[Test] Printing without pop up
printผ่าน os.startfile() มันทำให้ pdf reader ui มันเด้งขึ้นมาอาจจะ interupt การทำงานของผู้คน
</commit_message>
<xml_diff>
--- a/projects/Finance/inv_example.xlsx
+++ b/projects/Finance/inv_example.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BCP_27\Documents\GitHub\Python\projects\Finance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57FB9990-8FCD-4991-BE16-899AC7E34839}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{330DDDFB-F73F-4A9F-8CD6-E6DEA7D76750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6735" yWindow="2325" windowWidth="19425" windowHeight="10815" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2400" yWindow="870" windowWidth="19425" windowHeight="10815" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,18 +28,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="4">
   <si>
     <t>INVOICE_NO</t>
   </si>
   <si>
-    <t>B0183-W05-2408280037</t>
+    <t>B0183-W35-2408280026</t>
   </si>
   <si>
-    <t>B0183-W05-2408280038</t>
+    <t>B0183-W02-2408280011</t>
   </si>
   <si>
-    <t>B0183-W35-2408280025</t>
+    <t>B0183-W35-2408280027</t>
   </si>
 </sst>
 </file>
@@ -270,7 +270,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="21.85546875" customWidth="1"/>
@@ -288,11 +288,26 @@
     </row>
     <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
save update autopage shopee
shopee เปลี่ยน ui อีกแล้ว
</commit_message>
<xml_diff>
--- a/projects/Finance/inv_example.xlsx
+++ b/projects/Finance/inv_example.xlsx
@@ -1,24 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BCP_27\Documents\GitHub\Python\projects\Finance\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{330DDDFB-F73F-4A9F-8CD6-E6DEA7D76750}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="Calc"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="2400" yWindow="870" windowWidth="19425" windowHeight="10815" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$A$11</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet1!$A$1:$A$11</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -28,31 +23,55 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="4">
-  <si>
-    <t>INVOICE_NO</t>
-  </si>
-  <si>
-    <t>B0183-W35-2408280026</t>
-  </si>
-  <si>
-    <t>B0183-W02-2408280011</t>
-  </si>
-  <si>
-    <t>B0183-W35-2408280027</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+  <si>
+    <t xml:space="preserve">INVOICE_NO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B0183-W05-2408280044</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B0183-W35-2408280034</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B0183-W05-2408280045</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B0183-W35-2408280035</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B0183-W05-2408280046</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="General"/>
+  </numFmts>
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="222"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
     </font>
   </fonts>
   <fills count="2">
@@ -64,7 +83,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
@@ -72,77 +91,126 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="20">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  <cellXfs count="3">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
 </styleSheet>
 </file>
 
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="44546A"/>
+        <a:srgbClr val="44546a"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E7E6E6"/>
+        <a:srgbClr val="e7e6e6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4472C4"/>
+        <a:srgbClr val="4472c4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="ED7D31"/>
+        <a:srgbClr val="ed7d31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="A5A5A5"/>
+        <a:srgbClr val="a5a5a5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="FFC000"/>
+        <a:srgbClr val="ffc000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="5B9BD5"/>
+        <a:srgbClr val="5b9bd5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="70AD47"/>
+        <a:srgbClr val="70ad47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0563C1"/>
+        <a:srgbClr val="0563c1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="954F72"/>
+        <a:srgbClr val="954f72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -174,7 +242,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -198,7 +266,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -258,62 +326,69 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
-          <a:tileRect/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:A11"/>
+  <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="21.85546875" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.68"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
-      <c r="A2" t="s">
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
-      <c r="A3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1">
-      <c r="A4" t="s">
+    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:1">
-      <c r="A5" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1">
-      <c r="A6" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1">
-      <c r="A7" t="s">
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
     </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <autoFilter ref="A1:A11" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:A11"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>